<commit_message>
Tercero commit, se agrega la formula que va desde efectiva a nominal
</commit_message>
<xml_diff>
--- a/libreria-financiera.xlsx
+++ b/libreria-financiera.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/estebanmolina/Library/Mobile Documents/com~apple~CloudDocs/Ejercicios/02-Taller/P01-libreria-lambda/mi-construccion/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4D539C70-9A35-354C-9E9C-799F7D332396}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ABF17000-F816-A841-A444-B39D95FE7EB7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="21680" xr2:uid="{4EBB39A8-7C5E-6649-AA0E-B1C9F4122819}"/>
   </bookViews>
@@ -18,6 +18,7 @@
   </sheets>
   <definedNames>
     <definedName name="DatosExternos_8" localSheetId="0" hidden="1">Prueba!$A$1:$G$40</definedName>
+    <definedName name="TES_NOMINAL_TEA" comment="De efectiva a nominal">_xlfn.LAMBDA(_xlpm.i,_xlpm.m,IF(_xlpm.m &lt;= 0, NA(), _xlpm.m * ((1 + _xlpm.i) ^ (1 / _xlpm.m) - 1)))</definedName>
     <definedName name="TES_TEA_NOMINAL" comment="De nominal a efectiva">_xlfn.LAMBDA(_xlpm.m,_xlpm.j,IF(_xlpm.m &lt;= 0, NA(), ((1 + _xlpm.j / _xlpm.m) ^ _xlpm.m) - 1))</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
@@ -590,7 +591,7 @@
   <autoFilter ref="A1:G40" xr:uid="{B59D99B0-A4F5-7C4A-B4FA-40046C556F9E}">
     <filterColumn colId="1">
       <filters>
-        <filter val="TES_TEA_NOMINAL"/>
+        <filter val="TES_NOMINAL_TEA"/>
       </filters>
     </filterColumn>
   </autoFilter>
@@ -953,7 +954,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{503B5955-F743-A84A-8AAF-65C450073476}">
-  <dimension ref="A1:N40"/>
+  <dimension ref="A1:N41"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="5.1640625" bestFit="1" customWidth="1"/>
@@ -988,7 +989,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:14" hidden="1" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
         <v>91</v>
       </c>
@@ -1010,20 +1011,12 @@
       <c r="G2" s="1" t="s">
         <v>94</v>
       </c>
-      <c r="J2" s="2" cm="1">
-        <f t="array" ref="J2:K2">_xlfn.TEXTSPLIT(Base[[#This Row],[argumentos]],";")*1</f>
-        <v>0.12</v>
-      </c>
-      <c r="K2" s="2">
-        <v>12</v>
-      </c>
-      <c r="M2" s="2" cm="1">
-        <f t="array" ref="M2">TES_TEA_NOMINAL(K2,J2)</f>
-        <v>0.12682503013196977</v>
-      </c>
+      <c r="J2" s="2"/>
+      <c r="K2" s="2"/>
+      <c r="M2" s="2"/>
       <c r="N2" s="2"/>
     </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:14" hidden="1" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
         <v>95</v>
       </c>
@@ -1045,20 +1038,12 @@
       <c r="G3" s="1" t="s">
         <v>97</v>
       </c>
-      <c r="J3" s="2" cm="1">
-        <f t="array" ref="J3:K3">_xlfn.TEXTSPLIT(Base[[#This Row],[argumentos]],";")*1</f>
-        <v>5.0999999999999997E-2</v>
-      </c>
-      <c r="K3" s="2">
-        <v>12</v>
-      </c>
-      <c r="M3" s="2" cm="1">
-        <f t="array" ref="M3">TES_TEA_NOMINAL(K3,J3)</f>
-        <v>5.220917603681996E-2</v>
-      </c>
+      <c r="J3" s="2"/>
+      <c r="K3" s="2"/>
+      <c r="M3" s="2"/>
       <c r="N3" s="2"/>
     </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:14" hidden="1" x14ac:dyDescent="0.2">
       <c r="A4" s="1" t="s">
         <v>98</v>
       </c>
@@ -1080,20 +1065,12 @@
       <c r="G4" s="1" t="s">
         <v>100</v>
       </c>
-      <c r="J4" s="2" cm="1">
-        <f t="array" ref="J4:K4">_xlfn.TEXTSPLIT(Base[[#This Row],[argumentos]],";")*1</f>
-        <v>0.08</v>
-      </c>
-      <c r="K4" s="2">
-        <v>1</v>
-      </c>
-      <c r="M4" s="2" cm="1">
-        <f t="array" ref="M4">TES_TEA_NOMINAL(K4,J4)</f>
-        <v>8.0000000000000071E-2</v>
-      </c>
+      <c r="J4" s="2"/>
+      <c r="K4" s="2"/>
+      <c r="M4" s="2"/>
       <c r="N4" s="2"/>
     </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:14" hidden="1" x14ac:dyDescent="0.2">
       <c r="A5" s="1" t="s">
         <v>101</v>
       </c>
@@ -1115,20 +1092,12 @@
       <c r="G5" s="1" t="s">
         <v>103</v>
       </c>
-      <c r="J5" s="2" cm="1">
-        <f t="array" ref="J5:K5">_xlfn.TEXTSPLIT(Base[[#This Row],[argumentos]],";")*1</f>
-        <v>0.05</v>
-      </c>
-      <c r="K5" s="2">
-        <v>365</v>
-      </c>
-      <c r="M5" s="2" cm="1">
-        <f t="array" ref="M5">TES_TEA_NOMINAL(K5,J5)</f>
-        <v>5.1267496467422902E-2</v>
-      </c>
+      <c r="J5" s="2"/>
+      <c r="K5" s="2"/>
+      <c r="M5" s="2"/>
       <c r="N5" s="2"/>
     </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:14" hidden="1" x14ac:dyDescent="0.2">
       <c r="A6" s="1" t="s">
         <v>104</v>
       </c>
@@ -1150,20 +1119,12 @@
       <c r="G6" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="J6" s="2" cm="1">
-        <f t="array" ref="J6:K6">_xlfn.TEXTSPLIT(Base[[#This Row],[argumentos]],";")*1</f>
-        <v>0</v>
-      </c>
-      <c r="K6" s="2">
-        <v>12</v>
-      </c>
-      <c r="M6" s="2" cm="1">
-        <f t="array" ref="M6">TES_TEA_NOMINAL(K6,J6)</f>
-        <v>0</v>
-      </c>
+      <c r="J6" s="2"/>
+      <c r="K6" s="2"/>
+      <c r="M6" s="2"/>
       <c r="N6" s="2"/>
     </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:14" hidden="1" x14ac:dyDescent="0.2">
       <c r="A7" s="1" t="s">
         <v>106</v>
       </c>
@@ -1185,20 +1146,12 @@
       <c r="G7" s="1" t="s">
         <v>108</v>
       </c>
-      <c r="J7" s="2" cm="1">
-        <f t="array" ref="J7:K7">_xlfn.TEXTSPLIT(Base[[#This Row],[argumentos]],";")*1</f>
-        <v>0.12</v>
-      </c>
-      <c r="K7" s="2">
-        <v>0</v>
-      </c>
-      <c r="M7" s="2" t="e" cm="1">
-        <f t="array" ref="M7">TES_TEA_NOMINAL(K7,J7)</f>
-        <v>#N/A</v>
-      </c>
+      <c r="J7" s="2"/>
+      <c r="K7" s="2"/>
+      <c r="M7" s="2"/>
       <c r="N7" s="2"/>
     </row>
-    <row r="8" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:14" hidden="1" x14ac:dyDescent="0.2">
       <c r="A8" s="1" t="s">
         <v>109</v>
       </c>
@@ -1217,20 +1170,12 @@
       <c r="G8" s="1" t="s">
         <v>111</v>
       </c>
-      <c r="J8" s="2" cm="1">
-        <f t="array" ref="J8:K8">_xlfn.TEXTSPLIT(Base[[#This Row],[argumentos]],";")*1</f>
-        <v>0.12</v>
-      </c>
-      <c r="K8" s="2">
-        <v>-4</v>
-      </c>
-      <c r="M8" s="2" t="e" cm="1">
-        <f t="array" ref="M8">TES_TEA_NOMINAL(K8,J8)</f>
-        <v>#N/A</v>
-      </c>
+      <c r="J8" s="2"/>
+      <c r="K8" s="2"/>
+      <c r="M8" s="2"/>
       <c r="N8" s="2"/>
     </row>
-    <row r="9" spans="1:14" hidden="1" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A9" s="1" t="s">
         <v>33</v>
       </c>
@@ -1252,8 +1197,19 @@
       <c r="G9" s="1" t="s">
         <v>37</v>
       </c>
-    </row>
-    <row r="10" spans="1:14" hidden="1" x14ac:dyDescent="0.2">
+      <c r="I9" s="2" cm="1">
+        <f t="array" ref="I9:J9">_xlfn.TEXTSPLIT(Base[[#This Row],[argumentos]],";")*1</f>
+        <v>0.126825030131969</v>
+      </c>
+      <c r="J9" s="2">
+        <v>12</v>
+      </c>
+      <c r="L9" s="2" cm="1">
+        <f t="array" ref="L9">TES_NOMINAL_TEA(I9,J9)</f>
+        <v>0.12000000000000011</v>
+      </c>
+    </row>
+    <row r="10" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A10" s="1" t="s">
         <v>38</v>
       </c>
@@ -1275,8 +1231,19 @@
       <c r="G10" s="1" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="11" spans="1:14" hidden="1" x14ac:dyDescent="0.2">
+      <c r="I10" s="2" cm="1">
+        <f t="array" ref="I10:J10">_xlfn.TEXTSPLIT(Base[[#This Row],[argumentos]],";")*1</f>
+        <v>0.06</v>
+      </c>
+      <c r="J10" s="2">
+        <v>4</v>
+      </c>
+      <c r="L10" s="2" cm="1">
+        <f t="array" ref="L10">TES_NOMINAL_TEA(I10,J10)</f>
+        <v>5.8695384674637197E-2</v>
+      </c>
+    </row>
+    <row r="11" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A11" s="1" t="s">
         <v>41</v>
       </c>
@@ -1297,6 +1264,17 @@
       </c>
       <c r="G11" s="1" t="s">
         <v>44</v>
+      </c>
+      <c r="I11" s="2" cm="1">
+        <f t="array" ref="I11:J11">_xlfn.TEXTSPLIT(Base[[#This Row],[argumentos]],";")*1</f>
+        <v>-1</v>
+      </c>
+      <c r="J11" s="2">
+        <v>12</v>
+      </c>
+      <c r="L11" s="2" cm="1">
+        <f t="array" ref="L11">TES_NOMINAL_TEA(I11,J11)</f>
+        <v>-12</v>
       </c>
     </row>
     <row r="12" spans="1:14" hidden="1" x14ac:dyDescent="0.2">
@@ -1321,6 +1299,16 @@
       <c r="G12" s="1" t="s">
         <v>48</v>
       </c>
+      <c r="I12" s="2" cm="1">
+        <f t="array" ref="I12:K12">-_xlfn.TEXTSPLIT(Base[[#This Row],[argumentos]],";")</f>
+        <v>-0.06</v>
+      </c>
+      <c r="J12">
+        <v>-360</v>
+      </c>
+      <c r="K12">
+        <v>-30</v>
+      </c>
     </row>
     <row r="13" spans="1:14" hidden="1" x14ac:dyDescent="0.2">
       <c r="A13" s="1" t="s">
@@ -1344,6 +1332,16 @@
       <c r="G13" s="1" t="s">
         <v>51</v>
       </c>
+      <c r="I13" s="2" cm="1">
+        <f t="array" ref="I13:K13">-_xlfn.TEXTSPLIT(Base[[#This Row],[argumentos]],";")</f>
+        <v>-5.0000000000000001E-3</v>
+      </c>
+      <c r="J13">
+        <v>-30</v>
+      </c>
+      <c r="K13">
+        <v>-360</v>
+      </c>
     </row>
     <row r="14" spans="1:14" hidden="1" x14ac:dyDescent="0.2">
       <c r="A14" s="1" t="s">
@@ -1367,6 +1365,16 @@
       <c r="G14" s="1" t="s">
         <v>55</v>
       </c>
+      <c r="I14" s="2" cm="1">
+        <f t="array" ref="I14:K14">-_xlfn.TEXTSPLIT(Base[[#This Row],[argumentos]],";")</f>
+        <v>-0.06</v>
+      </c>
+      <c r="J14">
+        <v>-360</v>
+      </c>
+      <c r="K14">
+        <v>-360</v>
+      </c>
     </row>
     <row r="15" spans="1:14" hidden="1" x14ac:dyDescent="0.2">
       <c r="A15" s="1" t="s">
@@ -1390,6 +1398,16 @@
       <c r="G15" s="1" t="s">
         <v>58</v>
       </c>
+      <c r="I15" s="2" cm="1">
+        <f t="array" ref="I15:K15">-_xlfn.TEXTSPLIT(Base[[#This Row],[argumentos]],";")</f>
+        <v>-0.06</v>
+      </c>
+      <c r="J15">
+        <v>0</v>
+      </c>
+      <c r="K15">
+        <v>-30</v>
+      </c>
     </row>
     <row r="16" spans="1:14" hidden="1" x14ac:dyDescent="0.2">
       <c r="A16" s="1" t="s">
@@ -1413,8 +1431,21 @@
       <c r="G16" s="1" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="17" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+      <c r="I16" s="2" cm="1">
+        <f t="array" ref="I16:L16">-_xlfn.TEXTSPLIT(Base[[#This Row],[argumentos]],";")</f>
+        <v>-100000</v>
+      </c>
+      <c r="J16">
+        <v>-5.0999999999999997E-2</v>
+      </c>
+      <c r="K16">
+        <v>-360</v>
+      </c>
+      <c r="L16">
+        <v>-30</v>
+      </c>
+    </row>
+    <row r="17" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A17" s="1" t="s">
         <v>10</v>
       </c>
@@ -1436,8 +1467,21 @@
       <c r="G17" s="1" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="18" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+      <c r="I17" s="2" cm="1">
+        <f t="array" ref="I17:L17">-_xlfn.TEXTSPLIT(Base[[#This Row],[argumentos]],";")</f>
+        <v>-100000</v>
+      </c>
+      <c r="J17">
+        <v>-5.0999999999999997E-2</v>
+      </c>
+      <c r="K17">
+        <v>-360</v>
+      </c>
+      <c r="L17">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A18" s="1" t="s">
         <v>12</v>
       </c>
@@ -1459,8 +1503,21 @@
       <c r="G18" s="1" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="19" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+      <c r="I18" s="2" cm="1">
+        <f t="array" ref="I18:L18">-_xlfn.TEXTSPLIT(Base[[#This Row],[argumentos]],";")</f>
+        <v>-50000</v>
+      </c>
+      <c r="J18">
+        <v>-4.7500000000000001E-2</v>
+      </c>
+      <c r="K18">
+        <v>-45</v>
+      </c>
+      <c r="L18">
+        <v>-30</v>
+      </c>
+    </row>
+    <row r="19" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A19" s="1" t="s">
         <v>15</v>
       </c>
@@ -1482,8 +1539,21 @@
       <c r="G19" s="1" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="20" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+      <c r="I19" s="2" cm="1">
+        <f t="array" ref="I19:L19">-_xlfn.TEXTSPLIT(Base[[#This Row],[argumentos]],";")</f>
+        <v>-50000</v>
+      </c>
+      <c r="J19">
+        <v>-4.7500000000000001E-2</v>
+      </c>
+      <c r="K19">
+        <v>-20</v>
+      </c>
+      <c r="L19">
+        <v>-30</v>
+      </c>
+    </row>
+    <row r="20" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A20" s="1" t="s">
         <v>17</v>
       </c>
@@ -1505,8 +1575,21 @@
       <c r="G20" s="1" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="21" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+      <c r="I20" s="2" cm="1">
+        <f t="array" ref="I20:L20">-_xlfn.TEXTSPLIT(Base[[#This Row],[argumentos]],";")</f>
+        <v>-250000</v>
+      </c>
+      <c r="J20">
+        <v>-5.2499999999999998E-2</v>
+      </c>
+      <c r="K20">
+        <v>-181</v>
+      </c>
+      <c r="L20">
+        <v>-90</v>
+      </c>
+    </row>
+    <row r="21" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A21" s="1" t="s">
         <v>19</v>
       </c>
@@ -1528,8 +1611,24 @@
       <c r="G21" s="1" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="22" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+      <c r="I21" s="2" cm="1">
+        <f t="array" ref="I21:M21">-_xlfn.TEXTSPLIT(Base[[#This Row],[argumentos]],";")</f>
+        <v>-250000</v>
+      </c>
+      <c r="J21">
+        <v>-5.2499999999999998E-2</v>
+      </c>
+      <c r="K21">
+        <v>-365</v>
+      </c>
+      <c r="L21">
+        <v>-90</v>
+      </c>
+      <c r="M21">
+        <v>-365</v>
+      </c>
+    </row>
+    <row r="22" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A22" s="1" t="s">
         <v>21</v>
       </c>
@@ -1551,8 +1650,21 @@
       <c r="G22" s="1" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="23" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+      <c r="I22" s="2" cm="1">
+        <f t="array" ref="I22:L22">-_xlfn.TEXTSPLIT(Base[[#This Row],[argumentos]],";")</f>
+        <v>-100000</v>
+      </c>
+      <c r="J22">
+        <v>0</v>
+      </c>
+      <c r="K22">
+        <v>-360</v>
+      </c>
+      <c r="L22">
+        <v>-30</v>
+      </c>
+    </row>
+    <row r="23" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A23" s="1" t="s">
         <v>24</v>
       </c>
@@ -1574,8 +1686,21 @@
       <c r="G23" s="1" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="24" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+      <c r="I23" s="2" cm="1">
+        <f t="array" ref="I23:L23">-_xlfn.TEXTSPLIT(Base[[#This Row],[argumentos]],";")</f>
+        <v>-100000</v>
+      </c>
+      <c r="J23">
+        <v>-0.05</v>
+      </c>
+      <c r="K23">
+        <v>0</v>
+      </c>
+      <c r="L23">
+        <v>-30</v>
+      </c>
+    </row>
+    <row r="24" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A24" s="1" t="s">
         <v>26</v>
       </c>
@@ -1597,8 +1722,21 @@
       <c r="G24" s="1" t="s">
         <v>29</v>
       </c>
-    </row>
-    <row r="25" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+      <c r="I24" s="2" cm="1">
+        <f t="array" ref="I24:L24">-_xlfn.TEXTSPLIT(Base[[#This Row],[argumentos]],";")</f>
+        <v>-100000</v>
+      </c>
+      <c r="J24">
+        <v>-0.05</v>
+      </c>
+      <c r="K24">
+        <v>5</v>
+      </c>
+      <c r="L24">
+        <v>-30</v>
+      </c>
+    </row>
+    <row r="25" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A25" s="1" t="s">
         <v>30</v>
       </c>
@@ -1620,8 +1758,24 @@
       <c r="G25" s="1" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="26" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+      <c r="I25" s="2" cm="1">
+        <f t="array" ref="I25:M25">-_xlfn.TEXTSPLIT(Base[[#This Row],[argumentos]],";")</f>
+        <v>-100000</v>
+      </c>
+      <c r="J25">
+        <v>-0.05</v>
+      </c>
+      <c r="K25">
+        <v>-360</v>
+      </c>
+      <c r="L25">
+        <v>-30</v>
+      </c>
+      <c r="M25">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A26" s="1" t="s">
         <v>69</v>
       </c>
@@ -1643,8 +1797,18 @@
       <c r="G26" s="1" t="s">
         <v>72</v>
       </c>
-    </row>
-    <row r="27" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+      <c r="I26" s="2" cm="1">
+        <f t="array" ref="I26:K26">-_xlfn.TEXTSPLIT(Base[[#This Row],[argumentos]],";")</f>
+        <v>-100000</v>
+      </c>
+      <c r="J26">
+        <v>-105000</v>
+      </c>
+      <c r="K26">
+        <v>-360</v>
+      </c>
+    </row>
+    <row r="27" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A27" s="1" t="s">
         <v>73</v>
       </c>
@@ -1666,8 +1830,18 @@
       <c r="G27" s="1" t="s">
         <v>75</v>
       </c>
-    </row>
-    <row r="28" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+      <c r="I27" s="2" cm="1">
+        <f t="array" ref="I27:K27">-_xlfn.TEXTSPLIT(Base[[#This Row],[argumentos]],";")</f>
+        <v>-100000</v>
+      </c>
+      <c r="J27">
+        <v>-105000</v>
+      </c>
+      <c r="K27">
+        <v>-180</v>
+      </c>
+    </row>
+    <row r="28" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A28" s="1" t="s">
         <v>76</v>
       </c>
@@ -1689,8 +1863,21 @@
       <c r="G28" s="1" t="s">
         <v>78</v>
       </c>
-    </row>
-    <row r="29" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+      <c r="I28" s="2" cm="1">
+        <f t="array" ref="I28:L28">-_xlfn.TEXTSPLIT(Base[[#This Row],[argumentos]],";")</f>
+        <v>-100000</v>
+      </c>
+      <c r="J28">
+        <v>-101000</v>
+      </c>
+      <c r="K28">
+        <v>-30</v>
+      </c>
+      <c r="L28">
+        <v>-365</v>
+      </c>
+    </row>
+    <row r="29" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A29" s="1" t="s">
         <v>79</v>
       </c>
@@ -1712,8 +1899,18 @@
       <c r="G29" s="1" t="s">
         <v>81</v>
       </c>
-    </row>
-    <row r="30" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+      <c r="I29" s="2" cm="1">
+        <f t="array" ref="I29:K29">-_xlfn.TEXTSPLIT(Base[[#This Row],[argumentos]],";")</f>
+        <v>-100000</v>
+      </c>
+      <c r="J29">
+        <v>-100000</v>
+      </c>
+      <c r="K29">
+        <v>-90</v>
+      </c>
+    </row>
+    <row r="30" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A30" s="1" t="s">
         <v>82</v>
       </c>
@@ -1735,8 +1932,18 @@
       <c r="G30" s="1" t="s">
         <v>84</v>
       </c>
-    </row>
-    <row r="31" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+      <c r="I30" s="2" cm="1">
+        <f t="array" ref="I30:K30">-_xlfn.TEXTSPLIT(Base[[#This Row],[argumentos]],";")</f>
+        <v>-100000</v>
+      </c>
+      <c r="J30">
+        <v>-98000</v>
+      </c>
+      <c r="K30">
+        <v>-90</v>
+      </c>
+    </row>
+    <row r="31" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A31" s="1" t="s">
         <v>85</v>
       </c>
@@ -1758,8 +1965,18 @@
       <c r="G31" s="1" t="s">
         <v>87</v>
       </c>
-    </row>
-    <row r="32" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+      <c r="I31" s="2" cm="1">
+        <f t="array" ref="I31:K31">-_xlfn.TEXTSPLIT(Base[[#This Row],[argumentos]],";")</f>
+        <v>0</v>
+      </c>
+      <c r="J31">
+        <v>-1000</v>
+      </c>
+      <c r="K31">
+        <v>-90</v>
+      </c>
+    </row>
+    <row r="32" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A32" s="1" t="s">
         <v>88</v>
       </c>
@@ -1781,8 +1998,18 @@
       <c r="G32" s="1" t="s">
         <v>90</v>
       </c>
-    </row>
-    <row r="33" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+      <c r="I32" s="2" cm="1">
+        <f t="array" ref="I32:K32">-_xlfn.TEXTSPLIT(Base[[#This Row],[argumentos]],";")</f>
+        <v>-100000</v>
+      </c>
+      <c r="J32">
+        <v>-105000</v>
+      </c>
+      <c r="K32">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
       <c r="A33" s="1" t="s">
         <v>59</v>
       </c>
@@ -1804,8 +2031,15 @@
       <c r="G33" s="1" t="s">
         <v>62</v>
       </c>
-    </row>
-    <row r="34" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+      <c r="I33" s="2" cm="1">
+        <f t="array" ref="I33:J33">-_xlfn.TEXTSPLIT(Base[[#This Row],[argumentos]],";")</f>
+        <v>-5.0999999999999997E-2</v>
+      </c>
+      <c r="J33">
+        <v>-1.2E-2</v>
+      </c>
+    </row>
+    <row r="34" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
       <c r="A34" s="1" t="s">
         <v>63</v>
       </c>
@@ -1827,8 +2061,15 @@
       <c r="G34" s="1" t="s">
         <v>65</v>
       </c>
-    </row>
-    <row r="35" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+      <c r="I34" s="2" cm="1">
+        <f t="array" ref="I34:J34">-_xlfn.TEXTSPLIT(Base[[#This Row],[argumentos]],";")</f>
+        <v>-0.02</v>
+      </c>
+      <c r="J34">
+        <v>-0.05</v>
+      </c>
+    </row>
+    <row r="35" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
       <c r="A35" s="1" t="s">
         <v>66</v>
       </c>
@@ -1850,8 +2091,15 @@
       <c r="G35" s="1" t="s">
         <v>68</v>
       </c>
-    </row>
-    <row r="36" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+      <c r="I35" s="2" cm="1">
+        <f t="array" ref="I35:J35">-_xlfn.TEXTSPLIT(Base[[#This Row],[argumentos]],";")</f>
+        <v>-0.05</v>
+      </c>
+      <c r="J35">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="36" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
       <c r="A36" s="1" t="s">
         <v>112</v>
       </c>
@@ -1873,8 +2121,21 @@
       <c r="G36" s="1" t="s">
         <v>116</v>
       </c>
-    </row>
-    <row r="37" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+      <c r="I36" s="2" t="e" cm="1">
+        <f t="array" ref="I36:L36">-_xlfn.TEXTSPLIT(Base[[#This Row],[argumentos]],";")</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="J36" t="e">
+        <v>#VALUE!</v>
+      </c>
+      <c r="K36" t="e">
+        <v>#VALUE!</v>
+      </c>
+      <c r="L36" t="e">
+        <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="37" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
       <c r="A37" s="1" t="s">
         <v>117</v>
       </c>
@@ -1896,8 +2157,15 @@
       <c r="G37" s="1" t="s">
         <v>119</v>
       </c>
-    </row>
-    <row r="38" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+      <c r="I37" s="2" t="e" cm="1">
+        <f t="array" ref="I37:J37">-_xlfn.TEXTSPLIT(Base[[#This Row],[argumentos]],";")</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="J37" t="e">
+        <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="38" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
       <c r="A38" s="1" t="s">
         <v>120</v>
       </c>
@@ -1919,8 +2187,15 @@
       <c r="G38" s="1" t="s">
         <v>122</v>
       </c>
-    </row>
-    <row r="39" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+      <c r="I38" s="2" t="e" cm="1">
+        <f t="array" ref="I38:J38">-_xlfn.TEXTSPLIT(Base[[#This Row],[argumentos]],";")</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="J38" t="e">
+        <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="39" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
       <c r="A39" s="1" t="s">
         <v>123</v>
       </c>
@@ -1942,8 +2217,15 @@
       <c r="G39" s="1" t="s">
         <v>125</v>
       </c>
-    </row>
-    <row r="40" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+      <c r="I39" s="2" t="e" cm="1">
+        <f t="array" ref="I39:J39">-_xlfn.TEXTSPLIT(Base[[#This Row],[argumentos]],";")</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="J39" t="e">
+        <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="40" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
       <c r="A40" s="1" t="s">
         <v>126</v>
       </c>
@@ -1965,6 +2247,13 @@
       <c r="G40" s="1" t="s">
         <v>128</v>
       </c>
+      <c r="I40" s="2" t="e" cm="1">
+        <f t="array" ref="I40">-_xlfn.TEXTSPLIT(Base[[#This Row],[argumentos]],";")</f>
+        <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="41" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="I41" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Cuarto commit, para la fomrula de interes equivalente mismo interes en diferentes periodos de tiempo
</commit_message>
<xml_diff>
--- a/libreria-financiera.xlsx
+++ b/libreria-financiera.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/estebanmolina/Library/Mobile Documents/com~apple~CloudDocs/Ejercicios/02-Taller/P01-libreria-lambda/mi-construccion/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ABF17000-F816-A841-A444-B39D95FE7EB7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C89E3026-745B-FE48-AFAE-71C202B3BA12}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="21680" xr2:uid="{4EBB39A8-7C5E-6649-AA0E-B1C9F4122819}"/>
   </bookViews>
@@ -18,7 +18,8 @@
   </sheets>
   <definedNames>
     <definedName name="DatosExternos_8" localSheetId="0" hidden="1">Prueba!$A$1:$G$40</definedName>
-    <definedName name="TES_NOMINAL_TEA" comment="De efectiva a nominal">_xlfn.LAMBDA(_xlpm.i,_xlpm.m,IF(_xlpm.m &lt;= 0, NA(), _xlpm.m * ((1 + _xlpm.i) ^ (1 / _xlpm.m) - 1)))</definedName>
+    <definedName name="TES_NOMINAL_TEA" comment="De efectiva a nominal">_xlfn.LAMBDA(_xlpm.i,_xlpm.m,IF((_xlpm.m &lt;= 0) + (_xlpm.i &lt;= -1), NA(), _xlpm.m * ((1 + _xlpm.i) ^ (1 / _xlpm.m) - 1)))</definedName>
+    <definedName name="TES_TASA_EQUIV" comment="Convierte una tasa a su equivalente exacta en otro plazo">_xlfn.LAMBDA(_xlpm.tasa,_xlpm.dias_origen,_xlpm.dias_destino,IF((_xlpm.dias_origen &lt;= 0) + (_xlpm.tasa &lt;= -1), NA(), ((1 + _xlpm.tasa) ^ (_xlpm.dias_destino / _xlpm.dias_origen)) - 1))</definedName>
     <definedName name="TES_TEA_NOMINAL" comment="De nominal a efectiva">_xlfn.LAMBDA(_xlpm.m,_xlpm.j,IF(_xlpm.m &lt;= 0, NA(), ((1 + _xlpm.j / _xlpm.m) ^ _xlpm.m) - 1))</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
@@ -591,7 +592,7 @@
   <autoFilter ref="A1:G40" xr:uid="{B59D99B0-A4F5-7C4A-B4FA-40046C556F9E}">
     <filterColumn colId="1">
       <filters>
-        <filter val="TES_NOMINAL_TEA"/>
+        <filter val="TES_TASA_EQUIV"/>
       </filters>
     </filterColumn>
   </autoFilter>
@@ -954,7 +955,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{503B5955-F743-A84A-8AAF-65C450073476}">
-  <dimension ref="A1:N41"/>
+  <dimension ref="A1:M41"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="5.1640625" bestFit="1" customWidth="1"/>
@@ -966,7 +967,7 @@
     <col min="7" max="7" width="47.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -989,7 +990,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:14" hidden="1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
         <v>91</v>
       </c>
@@ -1013,10 +1014,10 @@
       </c>
       <c r="J2" s="2"/>
       <c r="K2" s="2"/>
+      <c r="L2" s="2"/>
       <c r="M2" s="2"/>
-      <c r="N2" s="2"/>
-    </row>
-    <row r="3" spans="1:14" hidden="1" x14ac:dyDescent="0.2">
+    </row>
+    <row r="3" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
         <v>95</v>
       </c>
@@ -1040,10 +1041,10 @@
       </c>
       <c r="J3" s="2"/>
       <c r="K3" s="2"/>
+      <c r="L3" s="2"/>
       <c r="M3" s="2"/>
-      <c r="N3" s="2"/>
-    </row>
-    <row r="4" spans="1:14" hidden="1" x14ac:dyDescent="0.2">
+    </row>
+    <row r="4" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A4" s="1" t="s">
         <v>98</v>
       </c>
@@ -1067,10 +1068,10 @@
       </c>
       <c r="J4" s="2"/>
       <c r="K4" s="2"/>
+      <c r="L4" s="2"/>
       <c r="M4" s="2"/>
-      <c r="N4" s="2"/>
-    </row>
-    <row r="5" spans="1:14" hidden="1" x14ac:dyDescent="0.2">
+    </row>
+    <row r="5" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A5" s="1" t="s">
         <v>101</v>
       </c>
@@ -1094,10 +1095,10 @@
       </c>
       <c r="J5" s="2"/>
       <c r="K5" s="2"/>
+      <c r="L5" s="2"/>
       <c r="M5" s="2"/>
-      <c r="N5" s="2"/>
-    </row>
-    <row r="6" spans="1:14" hidden="1" x14ac:dyDescent="0.2">
+    </row>
+    <row r="6" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A6" s="1" t="s">
         <v>104</v>
       </c>
@@ -1121,10 +1122,10 @@
       </c>
       <c r="J6" s="2"/>
       <c r="K6" s="2"/>
+      <c r="L6" s="2"/>
       <c r="M6" s="2"/>
-      <c r="N6" s="2"/>
-    </row>
-    <row r="7" spans="1:14" hidden="1" x14ac:dyDescent="0.2">
+    </row>
+    <row r="7" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A7" s="1" t="s">
         <v>106</v>
       </c>
@@ -1148,10 +1149,10 @@
       </c>
       <c r="J7" s="2"/>
       <c r="K7" s="2"/>
+      <c r="L7" s="2"/>
       <c r="M7" s="2"/>
-      <c r="N7" s="2"/>
-    </row>
-    <row r="8" spans="1:14" hidden="1" x14ac:dyDescent="0.2">
+    </row>
+    <row r="8" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A8" s="1" t="s">
         <v>109</v>
       </c>
@@ -1172,10 +1173,10 @@
       </c>
       <c r="J8" s="2"/>
       <c r="K8" s="2"/>
+      <c r="L8" s="2"/>
       <c r="M8" s="2"/>
-      <c r="N8" s="2"/>
-    </row>
-    <row r="9" spans="1:14" x14ac:dyDescent="0.2">
+    </row>
+    <row r="9" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A9" s="1" t="s">
         <v>33</v>
       </c>
@@ -1197,19 +1198,10 @@
       <c r="G9" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="I9" s="2" cm="1">
-        <f t="array" ref="I9:J9">_xlfn.TEXTSPLIT(Base[[#This Row],[argumentos]],";")*1</f>
-        <v>0.126825030131969</v>
-      </c>
-      <c r="J9" s="2">
-        <v>12</v>
-      </c>
-      <c r="L9" s="2" cm="1">
-        <f t="array" ref="L9">TES_NOMINAL_TEA(I9,J9)</f>
-        <v>0.12000000000000011</v>
-      </c>
-    </row>
-    <row r="10" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="I9" s="2"/>
+      <c r="J9" s="2"/>
+    </row>
+    <row r="10" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A10" s="1" t="s">
         <v>38</v>
       </c>
@@ -1231,19 +1223,10 @@
       <c r="G10" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="I10" s="2" cm="1">
-        <f t="array" ref="I10:J10">_xlfn.TEXTSPLIT(Base[[#This Row],[argumentos]],";")*1</f>
-        <v>0.06</v>
-      </c>
-      <c r="J10" s="2">
-        <v>4</v>
-      </c>
-      <c r="L10" s="2" cm="1">
-        <f t="array" ref="L10">TES_NOMINAL_TEA(I10,J10)</f>
-        <v>5.8695384674637197E-2</v>
-      </c>
-    </row>
-    <row r="11" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="I10" s="2"/>
+      <c r="J10" s="2"/>
+    </row>
+    <row r="11" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A11" s="1" t="s">
         <v>41</v>
       </c>
@@ -1265,19 +1248,10 @@
       <c r="G11" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="I11" s="2" cm="1">
-        <f t="array" ref="I11:J11">_xlfn.TEXTSPLIT(Base[[#This Row],[argumentos]],";")*1</f>
-        <v>-1</v>
-      </c>
-      <c r="J11" s="2">
-        <v>12</v>
-      </c>
-      <c r="L11" s="2" cm="1">
-        <f t="array" ref="L11">TES_NOMINAL_TEA(I11,J11)</f>
-        <v>-12</v>
-      </c>
-    </row>
-    <row r="12" spans="1:14" hidden="1" x14ac:dyDescent="0.2">
+      <c r="I11" s="2"/>
+      <c r="J11" s="2"/>
+    </row>
+    <row r="12" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A12" s="1" t="s">
         <v>45</v>
       </c>
@@ -1300,17 +1274,21 @@
         <v>48</v>
       </c>
       <c r="I12" s="2" cm="1">
-        <f t="array" ref="I12:K12">-_xlfn.TEXTSPLIT(Base[[#This Row],[argumentos]],";")</f>
-        <v>-0.06</v>
+        <f t="array" ref="I12:K12">_xlfn.TEXTSPLIT(Base[[#This Row],[argumentos]],";")*1</f>
+        <v>0.06</v>
       </c>
       <c r="J12">
-        <v>-360</v>
+        <v>360</v>
       </c>
       <c r="K12">
-        <v>-30</v>
-      </c>
-    </row>
-    <row r="13" spans="1:14" hidden="1" x14ac:dyDescent="0.2">
+        <v>30</v>
+      </c>
+      <c r="L12" s="2" cm="1">
+        <f t="array" ref="L12">TES_TASA_EQUIV(I12,J12,K12)</f>
+        <v>4.8675505653430484E-3</v>
+      </c>
+    </row>
+    <row r="13" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A13" s="1" t="s">
         <v>49</v>
       </c>
@@ -1333,17 +1311,21 @@
         <v>51</v>
       </c>
       <c r="I13" s="2" cm="1">
-        <f t="array" ref="I13:K13">-_xlfn.TEXTSPLIT(Base[[#This Row],[argumentos]],";")</f>
-        <v>-5.0000000000000001E-3</v>
+        <f t="array" ref="I13:K13">_xlfn.TEXTSPLIT(Base[[#This Row],[argumentos]],";")*1</f>
+        <v>5.0000000000000001E-3</v>
       </c>
       <c r="J13">
-        <v>-30</v>
+        <v>30</v>
       </c>
       <c r="K13">
-        <v>-360</v>
-      </c>
-    </row>
-    <row r="14" spans="1:14" hidden="1" x14ac:dyDescent="0.2">
+        <v>360</v>
+      </c>
+      <c r="L13" s="2" cm="1">
+        <f t="array" ref="L13">TES_TASA_EQUIV(I13,J13,K13)</f>
+        <v>6.1677811864497611E-2</v>
+      </c>
+    </row>
+    <row r="14" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A14" s="1" t="s">
         <v>52</v>
       </c>
@@ -1366,17 +1348,21 @@
         <v>55</v>
       </c>
       <c r="I14" s="2" cm="1">
-        <f t="array" ref="I14:K14">-_xlfn.TEXTSPLIT(Base[[#This Row],[argumentos]],";")</f>
-        <v>-0.06</v>
+        <f t="array" ref="I14:K14">_xlfn.TEXTSPLIT(Base[[#This Row],[argumentos]],";")*1</f>
+        <v>0.06</v>
       </c>
       <c r="J14">
-        <v>-360</v>
+        <v>360</v>
       </c>
       <c r="K14">
-        <v>-360</v>
-      </c>
-    </row>
-    <row r="15" spans="1:14" hidden="1" x14ac:dyDescent="0.2">
+        <v>360</v>
+      </c>
+      <c r="L14" s="2" cm="1">
+        <f t="array" ref="L14">TES_TASA_EQUIV(I14,J14,K14)</f>
+        <v>6.0000000000000053E-2</v>
+      </c>
+    </row>
+    <row r="15" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A15" s="1" t="s">
         <v>56</v>
       </c>
@@ -1399,17 +1385,21 @@
         <v>58</v>
       </c>
       <c r="I15" s="2" cm="1">
-        <f t="array" ref="I15:K15">-_xlfn.TEXTSPLIT(Base[[#This Row],[argumentos]],";")</f>
-        <v>-0.06</v>
+        <f t="array" ref="I15:K15">_xlfn.TEXTSPLIT(Base[[#This Row],[argumentos]],";")*1</f>
+        <v>0.06</v>
       </c>
       <c r="J15">
         <v>0</v>
       </c>
       <c r="K15">
-        <v>-30</v>
-      </c>
-    </row>
-    <row r="16" spans="1:14" hidden="1" x14ac:dyDescent="0.2">
+        <v>30</v>
+      </c>
+      <c r="L15" s="2" t="e" cm="1">
+        <f t="array" ref="L15">TES_TASA_EQUIV(I15,J15,K15)</f>
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="16" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A16" s="1" t="s">
         <v>6</v>
       </c>

</xml_diff>